<commit_message>
threat pool added to llm batch processing
</commit_message>
<xml_diff>
--- a/data/samples/test_addresses.xlsx
+++ b/data/samples/test_addresses.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rahulgupta/Documents/Coding/structured_address_ai_poc/data/samples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89AB5A13-B0CF-2C4B-8417-8A6870675EE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88CB6B26-4005-F646-8555-E17A3D2B643C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="1880" windowWidth="28040" windowHeight="17180" xr2:uid="{6F07F338-D208-7A41-832C-031358500E4C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="50">
   <si>
     <t>Addr_1</t>
   </si>
@@ -117,6 +117,75 @@
   </si>
   <si>
     <t>CN</t>
+  </si>
+  <si>
+    <t>Bahnhosfsstrrasse 15</t>
+  </si>
+  <si>
+    <t>6280 Zell am Ziller</t>
+  </si>
+  <si>
+    <t>Austria</t>
+  </si>
+  <si>
+    <t>AT</t>
+  </si>
+  <si>
+    <t>STRADA SA MARDONA CANTINE GEBELIAS</t>
+  </si>
+  <si>
+    <t>BARISARDO ITALIA</t>
+  </si>
+  <si>
+    <t>IE</t>
+  </si>
+  <si>
+    <t>Albertstraat 10</t>
+  </si>
+  <si>
+    <t>Antwerpen 2018</t>
+  </si>
+  <si>
+    <t>LT</t>
+  </si>
+  <si>
+    <t>PO BOX 247</t>
+  </si>
+  <si>
+    <t>HLUHLUWE</t>
+  </si>
+  <si>
+    <t>3960 SOUTH AFRICA</t>
+  </si>
+  <si>
+    <t>ZA</t>
+  </si>
+  <si>
+    <t>St 98</t>
+  </si>
+  <si>
+    <t>2nd Industry City</t>
+  </si>
+  <si>
+    <t>PO Box 1850</t>
+  </si>
+  <si>
+    <t>SA</t>
+  </si>
+  <si>
+    <t>Merve DUzkel</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>TEREZ KORUT55. C.EP.6. EMELET</t>
+  </si>
+  <si>
+    <t>1062 BUDAPEST, Hungary</t>
+  </si>
+  <si>
+    <t>ES</t>
   </si>
 </sst>
 </file>
@@ -488,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33DFABB4-F73B-044C-B027-E58C429E5B49}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
@@ -595,6 +664,95 @@
         <v>26</v>
       </c>
     </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>